<commit_message>
Atualiza scraping e dados de ensaio
</commit_message>
<xml_diff>
--- a/scraping/Dados_Daimer.xlsx
+++ b/scraping/Dados_Daimer.xlsx
@@ -21808,11 +21808,7 @@
           <t>Supervisor de Serviço de Campo</t>
         </is>
       </c>
-      <c r="P263" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
+      <c r="P263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">

</xml_diff>